<commit_message>
actualizacion login con cv
</commit_message>
<xml_diff>
--- a/MODELO_IMPORTAR.xlsx
+++ b/MODELO_IMPORTAR.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RGaristo\Desktop\mi-proyecto-python\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RGaristo\Desktop\IONOS\IONOS-GESTOR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE18BFF-AEEE-4A49-BC95-D509047D20B4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37436AA-D2A1-48E0-AA36-E11DC5502385}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Nombre</t>
   </si>
@@ -44,6 +44,21 @@
   </si>
   <si>
     <t>Fin</t>
+  </si>
+  <si>
+    <t>curso 1</t>
+  </si>
+  <si>
+    <t>Ricardo</t>
+  </si>
+  <si>
+    <t>99.8%</t>
+  </si>
+  <si>
+    <t>0/0/0</t>
+  </si>
+  <si>
+    <t>Borrar línea</t>
   </si>
 </sst>
 </file>
@@ -63,12 +78,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -84,11 +105,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" style="1" customWidth="1"/>
@@ -403,10 +427,11 @@
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -432,49 +457,71 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="6">
+        <v>46100</v>
+      </c>
+      <c r="F2" s="6">
+        <v>46101</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C16" s="3"/>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.25">

</xml_diff>